<commit_message>
corrected datum column in CoilSetup_ProtoMPEX.xlsx in Example 1
</commit_message>
<xml_diff>
--- a/Examples/Ex2 - ProtoMPEX/CoilSetup_ProtoMPEX.xlsx
+++ b/Examples/Ex2 - ProtoMPEX/CoilSetup_ProtoMPEX.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nfc\Documents\LDRD_RfNeutronSource\MagneticFieldGeometry\MagneticFieldCode\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nfc\Documents\MATLAB\MyRepos\MagneticFieldCode_Axisymmetric\Examples\Ex4 - ProtoMPEX_FluxMapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BD1D6C2-7D0C-48F6-BBED-0BE3E4A36E02}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C71F91C-BBC9-4664-8398-363576F7CC74}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{79EB1445-7373-446A-B7BC-60A0A49526E2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="5" xr2:uid="{79EB1445-7373-446A-B7BC-60A0A49526E2}"/>
   </bookViews>
   <sheets>
     <sheet name="conf_A" sheetId="1" r:id="rId1"/>
@@ -1011,7 +1011,7 @@
         <v>13</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>0.98809999999999998</v>
@@ -1050,7 +1050,7 @@
         <v>9</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3">
         <v>1.2981</v>
@@ -1080,7 +1080,7 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>1.6282000000000001</v>
@@ -1110,7 +1110,7 @@
         <v>12</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D5">
         <v>1.8642000000000001</v>
@@ -1140,7 +1140,7 @@
         <v>11</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D6">
         <v>2.1901999999999999</v>
@@ -1170,7 +1170,7 @@
         <v>13</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D7">
         <v>2.3881999999999999</v>
@@ -1200,7 +1200,7 @@
         <v>13</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D8">
         <v>2.9441999999999999</v>
@@ -1230,7 +1230,7 @@
         <v>13</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D9">
         <v>3.2201</v>
@@ -1260,7 +1260,7 @@
         <v>11</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D10">
         <v>3.4180999999999999</v>
@@ -1290,7 +1290,7 @@
         <v>8</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <v>3.7342</v>
@@ -1320,7 +1320,7 @@
         <v>8</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D12">
         <v>4.0480999999999998</v>
@@ -1350,7 +1350,7 @@
         <v>13</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D13">
         <v>4.3662000000000001</v>
@@ -1432,7 +1432,7 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>0.98809999999999998</v>
@@ -1471,7 +1471,7 @@
         <v>9</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3">
         <v>1.2981</v>
@@ -1501,7 +1501,7 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>1.6282000000000001</v>
@@ -1531,7 +1531,7 @@
         <v>12</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D5">
         <v>1.8642000000000001</v>
@@ -1561,7 +1561,7 @@
         <v>11</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D6">
         <v>2.1901999999999999</v>
@@ -1591,7 +1591,7 @@
         <v>8</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D7">
         <v>2.3881999999999999</v>
@@ -1621,7 +1621,7 @@
         <v>8</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D8">
         <v>2.9441999999999999</v>
@@ -1651,7 +1651,7 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D9">
         <v>3.2201</v>
@@ -1681,7 +1681,7 @@
         <v>8</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D10">
         <v>3.4180999999999999</v>
@@ -1711,7 +1711,7 @@
         <v>13</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <v>3.7342</v>
@@ -1741,7 +1741,7 @@
         <v>13</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D12">
         <v>4.0480999999999998</v>
@@ -1771,7 +1771,7 @@
         <v>8</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D13">
         <v>4.3662000000000001</v>
@@ -1853,7 +1853,7 @@
         <v>13</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>0.98809999999999998</v>
@@ -1892,7 +1892,7 @@
         <v>9</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3">
         <v>1.2981</v>
@@ -1922,7 +1922,7 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>1.6282000000000001</v>
@@ -1952,7 +1952,7 @@
         <v>12</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D5">
         <v>1.8642000000000001</v>
@@ -1982,7 +1982,7 @@
         <v>11</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D6">
         <v>2.1901999999999999</v>
@@ -2012,7 +2012,7 @@
         <v>13</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D7">
         <v>2.3881999999999999</v>
@@ -2042,7 +2042,7 @@
         <v>8</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D8">
         <v>2.9441999999999999</v>
@@ -2072,7 +2072,7 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D9">
         <v>3.1092</v>
@@ -2102,7 +2102,7 @@
         <v>13</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D10">
         <v>3.3887</v>
@@ -2132,7 +2132,7 @@
         <v>13</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <v>3.5918999999999999</v>
@@ -2162,7 +2162,7 @@
         <v>13</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D12">
         <v>3.7824</v>
@@ -2192,7 +2192,7 @@
         <v>13</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D13">
         <v>3.9729000000000001</v>
@@ -2222,7 +2222,7 @@
         <v>13</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D14">
         <v>4.2904</v>
@@ -2304,7 +2304,7 @@
         <v>12</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>0.98809999999999998</v>
@@ -2343,7 +2343,7 @@
         <v>9</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3">
         <v>1.2981</v>
@@ -2373,7 +2373,7 @@
         <v>10</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>1.6282000000000001</v>
@@ -2403,7 +2403,7 @@
         <v>10</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D5">
         <v>1.8642000000000001</v>
@@ -2433,7 +2433,7 @@
         <v>11</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D6">
         <v>2.1901999999999999</v>
@@ -2463,7 +2463,7 @@
         <v>12</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D7">
         <v>2.3881999999999999</v>
@@ -2493,7 +2493,7 @@
         <v>8</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D8">
         <v>2.9441999999999999</v>
@@ -2523,7 +2523,7 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D9">
         <v>3.1092</v>
@@ -2553,7 +2553,7 @@
         <v>13</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D10">
         <v>3.3887</v>
@@ -2583,7 +2583,7 @@
         <v>13</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <v>3.5918999999999999</v>
@@ -2613,7 +2613,7 @@
         <v>13</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D12">
         <v>3.7824</v>
@@ -2643,7 +2643,7 @@
         <v>13</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D13">
         <v>3.9729000000000001</v>
@@ -2673,7 +2673,7 @@
         <v>13</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D14">
         <v>4.2904</v>
@@ -2755,7 +2755,7 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>0.98809999999999998</v>
@@ -2794,7 +2794,7 @@
         <v>12</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3">
         <v>1.2981</v>
@@ -2824,7 +2824,7 @@
         <v>10</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>1.6282000000000001</v>
@@ -2854,7 +2854,7 @@
         <v>10</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D5">
         <v>1.8642000000000001</v>
@@ -2884,7 +2884,7 @@
         <v>11</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D6">
         <v>2.1901999999999999</v>
@@ -2914,7 +2914,7 @@
         <v>8</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D7">
         <v>2.3881999999999999</v>
@@ -2944,7 +2944,7 @@
         <v>8</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D8">
         <v>2.9441999999999999</v>
@@ -2974,7 +2974,7 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D9">
         <v>3.1092</v>
@@ -3004,7 +3004,7 @@
         <v>13</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D10">
         <v>3.3887</v>
@@ -3034,7 +3034,7 @@
         <v>13</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <v>3.5918999999999999</v>
@@ -3064,7 +3064,7 @@
         <v>13</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D12">
         <v>3.7824</v>
@@ -3094,7 +3094,7 @@
         <v>13</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D13">
         <v>3.9729000000000001</v>
@@ -3124,7 +3124,7 @@
         <v>13</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D14">
         <v>4.2904</v>
@@ -3206,7 +3206,7 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>0.98809999999999998</v>
@@ -3245,7 +3245,7 @@
         <v>9</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3">
         <v>1.2981</v>
@@ -3275,7 +3275,7 @@
         <v>10</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>1.6282000000000001</v>
@@ -3305,7 +3305,7 @@
         <v>10</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D5">
         <v>1.8642000000000001</v>
@@ -3335,7 +3335,7 @@
         <v>11</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D6">
         <v>2.1901999999999999</v>
@@ -3365,7 +3365,7 @@
         <v>8</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D7">
         <v>2.3881999999999999</v>
@@ -3395,7 +3395,7 @@
         <v>12</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D8">
         <v>2.9441999999999999</v>
@@ -3425,7 +3425,7 @@
         <v>12</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D9">
         <v>3.1092</v>
@@ -3455,7 +3455,7 @@
         <v>13</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D10">
         <v>3.3887</v>
@@ -3485,7 +3485,7 @@
         <v>13</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <v>3.5918999999999999</v>
@@ -3515,7 +3515,7 @@
         <v>13</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D12">
         <v>3.7824</v>
@@ -3545,7 +3545,7 @@
         <v>13</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D13">
         <v>3.9729000000000001</v>
@@ -3575,7 +3575,7 @@
         <v>13</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D14">
         <v>4.2904</v>

</xml_diff>